<commit_message>
Refresh EDA pipeline outputs and add app-level base metrics
- Re-run EDA Section A-E against current cleansed English subset.
- Update workbooks and bilingual conclusion PDF/PPT.
- Add build_app_base_metrics.py and config (metrics.json, benchmark_flagship.json).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/google play/reports/eda_section_a_workbook.xlsx
+++ b/google play/reports/eda_section_a_workbook.xlsx
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>3680</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="3">
@@ -453,7 +453,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>569</v>
+        <v>776</v>
       </c>
     </row>
     <row r="4">
@@ -464,7 +464,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>625</v>
+        <v>842</v>
       </c>
     </row>
     <row r="5">
@@ -475,7 +475,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>990</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="6">
@@ -486,7 +486,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>4305</v>
+        <v>5903</v>
       </c>
     </row>
   </sheetData>
@@ -546,28 +546,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ai.character.app</t>
+          <t>air.com.sgn.cookiejam.gp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AI Chat</t>
+          <t>Cookie Jam</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>894</v>
+        <v>91</v>
       </c>
       <c r="E2" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F2" t="n">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="H2" t="n">
-        <v>72</v>
+        <v>557</v>
       </c>
     </row>
     <row r="3">
@@ -576,28 +576,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>com.apple.atve.sony.appletv</t>
+          <t>com.disney.emojimatch_goo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Apple TV</t>
+          <t>Disney Emoji Blitz</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>341</v>
+        <v>155</v>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F3" t="n">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="G3" t="n">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="H3" t="n">
-        <v>71</v>
+        <v>528</v>
       </c>
     </row>
     <row r="4">
@@ -606,28 +606,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>com.bigwinepot.nwdn.international</t>
+          <t>com.dreamgames.royalkingdom</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Remini</t>
+          <t>Royal Kingdom</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>227</v>
+        <v>415</v>
       </c>
       <c r="E4" t="n">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="F4" t="n">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="G4" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="H4" t="n">
-        <v>133</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5">
@@ -636,28 +636,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>com.canva.editor</t>
+          <t>com.dreamgames.royalmatch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Canva:AI</t>
+          <t>Royal Match</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>54</v>
+        <v>208</v>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F5" t="n">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="H5" t="n">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6">
@@ -666,28 +666,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>com.duolingo</t>
+          <t>com.king.candycrushsaga</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Duolingo</t>
+          <t>Candy Crush Saga</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="G6" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="H6" t="n">
-        <v>547</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7">
@@ -696,28 +696,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>com.flyersoft.moonreaderp</t>
+          <t>com.king.candycrushsodasaga</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Moon+Reader Pro</t>
+          <t>Candy Crush Soda Saga</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="E7" t="n">
-        <v>88</v>
+        <v>45</v>
       </c>
       <c r="F7" t="n">
-        <v>129</v>
+        <v>48</v>
       </c>
       <c r="G7" t="n">
-        <v>207</v>
+        <v>52</v>
       </c>
       <c r="H7" t="n">
-        <v>527</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8">
@@ -726,28 +726,28 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>com.google.android.youtube</t>
+          <t>com.playrix.gardenscapes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Gardenscapes</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>245</v>
+        <v>171</v>
       </c>
       <c r="E8" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="G8" t="n">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="H8" t="n">
-        <v>240</v>
+        <v>319</v>
       </c>
     </row>
     <row r="9">
@@ -756,28 +756,28 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>com.qidian.Int.reader</t>
+          <t>com.playrix.homescapes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>WebNovel</t>
+          <t>Homescapes</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="E9" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="F9" t="n">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="G9" t="n">
-        <v>195</v>
+        <v>83</v>
       </c>
       <c r="H9" t="n">
-        <v>464</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10">
@@ -786,28 +786,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>com.twitter.android</t>
+          <t>com.rovio.angrybirdsfriends</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Angry Birds Friends</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>530</v>
+        <v>164</v>
       </c>
       <c r="E10" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="F10" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="G10" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="H10" t="n">
-        <v>220</v>
+        <v>370</v>
       </c>
     </row>
     <row r="11">
@@ -816,28 +816,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>com.zhiliaoapp.musically</t>
+          <t>com.rovio.dream</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Angry Birds Dream Blast</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>374</v>
+        <v>167</v>
       </c>
       <c r="E11" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="F11" t="n">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="G11" t="n">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="H11" t="n">
-        <v>253</v>
+        <v>477</v>
       </c>
     </row>
     <row r="12">
@@ -846,28 +846,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>jp.ne.ibis.ibispaint.app</t>
+          <t>dk.tactile.lilysgarden</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ibis Paint</t>
+          <t>Lily's Garden</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>120</v>
+        <v>203</v>
       </c>
       <c r="E12" t="n">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="F12" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G12" t="n">
-        <v>148</v>
+        <v>77</v>
       </c>
       <c r="H12" t="n">
-        <v>578</v>
+        <v>567</v>
       </c>
     </row>
     <row r="13">
@@ -876,28 +876,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>net.mbc.shahidTV</t>
+          <t>dk.tactile.mansionstory</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MBC Shahid</t>
+          <t>Penny &amp; Flo</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="E13" t="n">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="G13" t="n">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="H13" t="n">
-        <v>37</v>
+        <v>572</v>
       </c>
     </row>
     <row r="14">
@@ -906,28 +906,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>org.telegram.messenger</t>
+          <t>net.peakgames.amy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Telegram</t>
+          <t>Toy Blast</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>321</v>
+        <v>140</v>
       </c>
       <c r="E14" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="G14" t="n">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="H14" t="n">
-        <v>240</v>
+        <v>460</v>
       </c>
     </row>
     <row r="15">
@@ -936,28 +936,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>voicerecorder.audiorecorder.voice</t>
+          <t>net.peakgames.toonblast</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Voice Recorder Audio Sound MP3</t>
+          <t>Toon Blast</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>33</v>
+        <v>216</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="G15" t="n">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="H15" t="n">
-        <v>600</v>
+        <v>373</v>
       </c>
     </row>
     <row r="18">
@@ -988,19 +988,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ai.character.app</t>
+          <t>air.com.sgn.cookiejam.gp</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AI Chat</t>
+          <t>Cookie Jam</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.472072072072072</v>
+        <v>4.08172531214529</v>
       </c>
       <c r="E19" t="n">
-        <v>1110</v>
+        <v>881</v>
       </c>
     </row>
     <row r="20">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>com.apple.atve.sony.appletv</t>
+          <t>com.disney.emojimatch_goo</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Apple TV</t>
+          <t>Disney Emoji Blitz</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.914772727272727</v>
+        <v>3.839632277834525</v>
       </c>
       <c r="E20" t="n">
-        <v>528</v>
+        <v>979</v>
       </c>
     </row>
     <row r="21">
@@ -1030,19 +1030,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>com.bigwinepot.nwdn.international</t>
+          <t>com.dreamgames.royalkingdom</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Remini</t>
+          <t>Royal Kingdom</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2.555819477434679</v>
+        <v>2.488940628637951</v>
       </c>
       <c r="E21" t="n">
-        <v>421</v>
+        <v>859</v>
       </c>
     </row>
     <row r="22">
@@ -1051,19 +1051,19 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>com.canva.editor</t>
+          <t>com.dreamgames.royalmatch</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Canva:AI</t>
+          <t>Royal Match</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>4.174603174603175</v>
+        <v>3.328947368421053</v>
       </c>
       <c r="E22" t="n">
-        <v>504</v>
+        <v>684</v>
       </c>
     </row>
     <row r="23">
@@ -1072,19 +1072,19 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>com.duolingo</t>
+          <t>com.king.candycrushsaga</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Duolingo</t>
+          <t>Candy Crush Saga</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.344783715012722</v>
+        <v>4.228070175438597</v>
       </c>
       <c r="E23" t="n">
-        <v>786</v>
+        <v>513</v>
       </c>
     </row>
     <row r="24">
@@ -1093,19 +1093,19 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>com.flyersoft.moonreaderp</t>
+          <t>com.king.candycrushsodasaga</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Moon+Reader Pro</t>
+          <t>Candy Crush Soda Saga</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3.767776777677768</v>
+        <v>3.967692307692307</v>
       </c>
       <c r="E24" t="n">
-        <v>1111</v>
+        <v>650</v>
       </c>
     </row>
     <row r="25">
@@ -1114,19 +1114,19 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>com.google.android.youtube</t>
+          <t>com.playrix.gardenscapes</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Gardenscapes</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2.966898954703833</v>
+        <v>3.482539682539683</v>
       </c>
       <c r="E25" t="n">
-        <v>574</v>
+        <v>630</v>
       </c>
     </row>
     <row r="26">
@@ -1135,19 +1135,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>com.qidian.Int.reader</t>
+          <t>com.playrix.homescapes</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>WebNovel</t>
+          <t>Homescapes</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>3.805467928496319</v>
+        <v>3.824404761904762</v>
       </c>
       <c r="E26" t="n">
-        <v>951</v>
+        <v>672</v>
       </c>
     </row>
     <row r="27">
@@ -1156,19 +1156,19 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>com.twitter.android</t>
+          <t>com.rovio.angrybirdsfriends</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Angry Birds Friends</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.301714285714286</v>
+        <v>3.59915611814346</v>
       </c>
       <c r="E27" t="n">
-        <v>875</v>
+        <v>711</v>
       </c>
     </row>
     <row r="28">
@@ -1177,19 +1177,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>com.zhiliaoapp.musically</t>
+          <t>com.rovio.dream</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Angry Birds Dream Blast</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.668449197860963</v>
+        <v>3.766944114149822</v>
       </c>
       <c r="E28" t="n">
-        <v>748</v>
+        <v>841</v>
       </c>
     </row>
     <row r="29">
@@ -1198,19 +1198,19 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>jp.ne.ibis.ibispaint.app</t>
+          <t>dk.tactile.lilysgarden</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ibis Paint</t>
+          <t>Lily's Garden</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4.037832310838446</v>
+        <v>3.73420260782347</v>
       </c>
       <c r="E29" t="n">
-        <v>978</v>
+        <v>997</v>
       </c>
     </row>
     <row r="30">
@@ -1219,19 +1219,19 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>net.mbc.shahidTV</t>
+          <t>dk.tactile.mansionstory</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MBC Shahid</t>
+          <t>Penny &amp; Flo</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.892561983471074</v>
+        <v>3.940162271805274</v>
       </c>
       <c r="E30" t="n">
-        <v>242</v>
+        <v>986</v>
       </c>
     </row>
     <row r="31">
@@ -1240,19 +1240,19 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>org.telegram.messenger</t>
+          <t>net.peakgames.amy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Telegram</t>
+          <t>Toy Blast</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2.744648318042814</v>
+        <v>3.888</v>
       </c>
       <c r="E31" t="n">
-        <v>654</v>
+        <v>750</v>
       </c>
     </row>
     <row r="32">
@@ -1261,19 +1261,19 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>voicerecorder.audiorecorder.voice</t>
+          <t>net.peakgames.toonblast</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Voice Recorder Audio Sound MP3</t>
+          <t>Toon Blast</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4.684133915574964</v>
+        <v>3.401524777636594</v>
       </c>
       <c r="E32" t="n">
-        <v>687</v>
+        <v>787</v>
       </c>
     </row>
   </sheetData>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10169</v>
+        <v>10940</v>
       </c>
     </row>
     <row r="3">
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>125.1738617366506</v>
+        <v>112.2530164533821</v>
       </c>
     </row>
     <row r="4">
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>129.3126972253494</v>
+        <v>122.1556412916507</v>
       </c>
     </row>
     <row r="5">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7">
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>333</v>
+        <v>300</v>
       </c>
     </row>
     <row r="8">
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>447</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9">
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>760</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -1450,13 +1450,13 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>153.2828804347826</v>
+        <v>165.659158521037</v>
       </c>
       <c r="D2" t="n">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="E2" t="n">
-        <v>3680</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="3">
@@ -1467,13 +1467,13 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>177.2583479789104</v>
+        <v>195.4690721649484</v>
       </c>
       <c r="D3" t="n">
-        <v>134</v>
+        <v>164</v>
       </c>
       <c r="E3" t="n">
-        <v>569</v>
+        <v>776</v>
       </c>
     </row>
     <row r="4">
@@ -1484,13 +1484,13 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>172.4096</v>
+        <v>177.312351543943</v>
       </c>
       <c r="D4" t="n">
-        <v>126</v>
+        <v>135.5</v>
       </c>
       <c r="E4" t="n">
-        <v>625</v>
+        <v>842</v>
       </c>
     </row>
     <row r="5">
@@ -1501,13 +1501,13 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>143.6525252525253</v>
+        <v>118.9230769230769</v>
       </c>
       <c r="D5" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
-        <v>990</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="6">
@@ -1518,13 +1518,13 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>83.15447154471545</v>
+        <v>69.54074199559545</v>
       </c>
       <c r="D6" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
-        <v>4305</v>
+        <v>5903</v>
       </c>
     </row>
   </sheetData>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>15405</v>
+        <v>16800</v>
       </c>
     </row>
     <row r="3">
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13806</v>
+        <v>15290</v>
       </c>
     </row>
     <row r="4">
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10169</v>
+        <v>10940</v>
       </c>
     </row>
   </sheetData>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1480971580293047</v>
+        <v>0.2937842778793418</v>
       </c>
     </row>
   </sheetData>
@@ -1703,10 +1703,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>3.220708761399053</v>
+        <v>3.824488739321771</v>
       </c>
       <c r="D2" t="n">
-        <v>8663</v>
+        <v>7726</v>
       </c>
     </row>
     <row r="3">
@@ -1717,10 +1717,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>2.839973439575033</v>
+        <v>3.317361543248289</v>
       </c>
       <c r="D3" t="n">
-        <v>1506</v>
+        <v>3214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>